<commit_message>
8. Driver excel changes done
</commit_message>
<xml_diff>
--- a/rabbit-web-app/public/sample_excels/driver_bulk_sample.xlsx
+++ b/rabbit-web-app/public/sample_excels/driver_bulk_sample.xlsx
@@ -398,31 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W11"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="28.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="23.83203125" customWidth="1"/>
-    <col min="15" max="15" width="26.83203125" customWidth="1"/>
-    <col min="16" max="16" width="17.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-    <col min="18" max="18" width="18.83203125" customWidth="1"/>
-    <col min="19" max="19" width="31.83203125" customWidth="1"/>
-    <col min="20" max="20" width="19.83203125" customWidth="1"/>
-    <col min="21" max="21" width="19.83203125" customWidth="1"/>
-    <col min="22" max="22" width="42.83203125" customWidth="1"/>
-    <col min="23" max="23" width="37.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -459,7 +434,7 @@
         <v>Country*</v>
       </c>
       <c r="L1" t="str">
-        <v>Postal Code</v>
+        <v>Zip Code</v>
       </c>
       <c r="M1" t="str">
         <v>License Number</v>
@@ -503,7 +478,7 @@
         <v>gurpreet.singh.driver@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>+1 555-234-8891</v>
+        <v>555-234-8891</v>
       </c>
       <c r="D2" t="str">
         <v>ACHA9999</v>
@@ -554,7 +529,7 @@
         <v>gurpreet.personal@gmail.com</v>
       </c>
       <c r="T2" t="str">
-        <v>+1 555-234-8890</v>
+        <v>555-234-8890</v>
       </c>
       <c r="U2" t="str">
         <v>View, Edit, Add</v>
@@ -574,7 +549,7 @@
         <v>rajesh.sharma.trucking@gmail.com</v>
       </c>
       <c r="C3" t="str">
-        <v>+1 555-345-9922</v>
+        <v>555-345-9922</v>
       </c>
       <c r="D3" t="str">
         <v>AQWSAS4323, BZ88BS77</v>
@@ -645,7 +620,7 @@
         <v>harpreet.kaur.freight@gmail.com</v>
       </c>
       <c r="C4" t="str">
-        <v>+1 555-456-1133</v>
+        <v>555-456-1133</v>
       </c>
       <c r="D4" t="str">
         <v>CH001, CH0014</v>
@@ -716,7 +691,7 @@
         <v>amit.patel.trans@gmail.com</v>
       </c>
       <c r="C5" t="str">
-        <v>+1 555-567-2244</v>
+        <v>555-567-2244</v>
       </c>
       <c r="D5" t="str">
         <v>CH0013</v>
@@ -767,7 +742,7 @@
         <v>amit.patel99@gmail.com</v>
       </c>
       <c r="T5" t="str">
-        <v>+1 555-567-2200</v>
+        <v>555-567-2200</v>
       </c>
       <c r="U5" t="str">
         <v>View</v>
@@ -787,7 +762,7 @@
         <v>jaswinder.sandhu.logistics@gmail.com</v>
       </c>
       <c r="C6" t="str">
-        <v>+1 555-678-3355</v>
+        <v>555-678-3355</v>
       </c>
       <c r="D6" t="str">
         <v>CH002, CH011</v>
@@ -858,7 +833,7 @@
         <v>vikram.malhotra.express@gmail.com</v>
       </c>
       <c r="C7" t="str">
-        <v>+1 555-789-4466</v>
+        <v>555-789-4466</v>
       </c>
       <c r="D7" t="str">
         <v>CH0020</v>
@@ -929,7 +904,7 @@
         <v>manpreet.singh.lines@gmail.com</v>
       </c>
       <c r="C8" t="str">
-        <v>+1 555-890-5577</v>
+        <v>555-890-5577</v>
       </c>
       <c r="D8" t="str">
         <v>CH003, CH012</v>
@@ -980,7 +955,7 @@
         <v/>
       </c>
       <c r="T8" t="str">
-        <v>+1 555-890-5500</v>
+        <v>555-890-5500</v>
       </c>
       <c r="U8" t="str">
         <v>View, Edit, Add</v>
@@ -1000,7 +975,7 @@
         <v>sunil.verma.carriers@gmail.com</v>
       </c>
       <c r="C9" t="str">
-        <v>+1 555-901-6688</v>
+        <v>555-901-6688</v>
       </c>
       <c r="D9" t="str">
         <v>CH013, CH016</v>
@@ -1071,7 +1046,7 @@
         <v>navjot.dhillon.transport@gmail.com</v>
       </c>
       <c r="C10" t="str">
-        <v>+1 555-012-7799</v>
+        <v>555-012-7799</v>
       </c>
       <c r="D10" t="str">
         <v>CH017, CH018, CH021</v>
@@ -1142,7 +1117,7 @@
         <v>deepak.choudhary.haul@gmail.com</v>
       </c>
       <c r="C11" t="str">
-        <v>+1 555-123-8800</v>
+        <v>555-123-8800</v>
       </c>
       <c r="D11" t="str">
         <v>DRY098JJHH, RMSS123, SMR2233</v>
@@ -1193,7 +1168,7 @@
         <v>deepak.ch@gmail.com</v>
       </c>
       <c r="T11" t="str">
-        <v>+1 555-123-8801</v>
+        <v>555-123-8801</v>
       </c>
       <c r="U11" t="str">
         <v>View, Edit, Add</v>

</xml_diff>